<commit_message>
rev.B : add PWM Ctrl
</commit_message>
<xml_diff>
--- a/Generate Files/BOM/247-616_Pi-CAN.xlsx
+++ b/Generate Files/BOM/247-616_Pi-CAN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin.cotton\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/247-616 (last) - Elaborer l integration et l installation de systemes ordines/Laboratoires/_Laboratoire3-Can/247-616_Pi-CAN-PCB/Generate Files/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5DC688C-43BA-44A1-8279-1DA85B198641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{7ABD1E47-55B8-446F-BC17-085BFAE5DBB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{727A9A75-CA73-4317-9FF2-FA4454268677}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37B24FDB-EB3D-4E0E-9FA8-8963631D87DA}"/>
+    <workbookView xWindow="1188" yWindow="228" windowWidth="19620" windowHeight="11352" xr2:uid="{47A388A6-04D0-47D7-9EEF-EE78C7524854}"/>
   </bookViews>
   <sheets>
     <sheet name="247-616_Pi-CAN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="120">
   <si>
     <t>LibRef</t>
   </si>
@@ -104,7 +104,7 @@
     <t>Capacitor type 1</t>
   </si>
   <si>
-    <t>C1, C2</t>
+    <t>C1, C2, C7</t>
   </si>
   <si>
     <t>Yageo</t>
@@ -131,7 +131,7 @@
     <t>Cap 10uF 0805</t>
   </si>
   <si>
-    <t>C3, C4</t>
+    <t>C3, C4, C8</t>
   </si>
   <si>
     <t>Samsung</t>
@@ -212,6 +212,48 @@
     <t>277-6163-ND</t>
   </si>
   <si>
+    <t>J_DC_JACK_2.5MM</t>
+  </si>
+  <si>
+    <t>694106301002</t>
+  </si>
+  <si>
+    <t>DC Barrel Connector 2.5mm</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>XKB Connection</t>
+  </si>
+  <si>
+    <t>DC-005-5A-2.5</t>
+  </si>
+  <si>
+    <t>C381115</t>
+  </si>
+  <si>
+    <t>P_HEADER_3POS</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>61300311121</t>
+  </si>
+  <si>
+    <t>Header 3pins single row, TH</t>
+  </si>
+  <si>
+    <t>P1, P2, P3, P5, P6</t>
+  </si>
+  <si>
+    <t>Würth Elektronik</t>
+  </si>
+  <si>
+    <t>732-5316-ND</t>
+  </si>
+  <si>
     <t>RES015</t>
   </si>
   <si>
@@ -260,7 +302,7 @@
     <t>Res 10k 1% 0603</t>
   </si>
   <si>
-    <t>R3, R5</t>
+    <t>R3, R5, R6, R7</t>
   </si>
   <si>
     <t>RC0603FR-0710KL</t>
@@ -320,16 +362,22 @@
     <t>U2</t>
   </si>
   <si>
-    <t>CMP-1595-00004-2</t>
+    <t>U_PCA9685PW</t>
   </si>
   <si>
     <t>PCA9685PW,112</t>
   </si>
   <si>
-    <t>16-Channel, 12-Bit PWM Fm+ I2C-Bus LED Controller, 2.3 to 5.5 V, -40 to 85 degC, 28-Pin TSSOP (SOT361-1), RoHS, Tape and Reel</t>
+    <t>16-Channel, 12-Bit PWM I2C-Bus LED Controller, 28-Pin TSSOP (SOT361-1)</t>
   </si>
   <si>
     <t>U3</t>
+  </si>
+  <si>
+    <t>NXP</t>
+  </si>
+  <si>
+    <t>568-8366-5-ND</t>
   </si>
   <si>
     <t>Y_XTAL_8MHz_HC49US</t>
@@ -356,7 +404,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -418,7 +466,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{67DA9B97-54FE-47BE-9B1C-7F5834DE8317}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -746,8 +796,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3226906E-65A5-484A-B7E6-A757345A2544}">
-  <dimension ref="A1:Q14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61FF1AED-653B-4547-A861-B058579B7014}">
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.21875" customWidth="1"/>
@@ -829,7 +879,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>20</v>
@@ -870,7 +920,7 @@
         <v>29</v>
       </c>
       <c r="D3" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>20</v>
@@ -1037,10 +1087,10 @@
         <v>60</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -1048,79 +1098,79 @@
         <v>24</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="2" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" s="1"/>
+        <v>64</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="C8" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D8" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="2" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="2" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="2" t="s">
         <v>71</v>
       </c>
+      <c r="B9" s="1"/>
       <c r="C9" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>22</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -1128,7 +1178,7 @@
         <v>24</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
@@ -1140,34 +1190,34 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="2" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
@@ -1179,144 +1229,154 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D11" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="2" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="2" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>89</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="B12" s="1"/>
       <c r="C12" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>92</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
+      <c r="K12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="2" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B13" s="1"/>
+        <v>95</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="C13" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D13" s="1">
         <v>1</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+        <v>99</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
+      <c r="K13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>101</v>
+      </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
+      <c r="Q13" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>103</v>
-      </c>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
@@ -1325,6 +1385,86 @@
         <v>48</v>
       </c>
     </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
first commit projet ESA v1
</commit_message>
<xml_diff>
--- a/Generate Files/BOM/247-616_Pi-CAN.xlsx
+++ b/Generate Files/BOM/247-616_Pi-CAN.xlsx
@@ -1521,4 +1521,284 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100195A0DC3D759E3489DFA9C5205E5B14C" ma:contentTypeVersion="18" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="c10faa181153c6f142d687ced5214bba">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557b78e-b540-44eb-8496-d55148e88a38" xmlns:ns3="cd07618e-4042-4e05-8059-9e82e303398b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b35beefd964c4cbe5e2adf78b7e80be7" ns2:_="" ns3:_="">
+    <xsd:import namespace="9557b78e-b540-44eb-8496-d55148e88a38"/>
+    <xsd:import namespace="cd07618e-4042-4e05-8059-9e82e303398b"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:date" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9557b78e-b540-44eb-8496-d55148e88a38" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="12" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="15" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="16" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7a0a163c-996e-4842-8c49-2f1fe733ec08" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="20" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="22" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="23" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="date" ma:index="24" nillable="true" ma:displayName="date" ma:format="DateOnly" ma:internalName="date">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="cd07618e-4042-4e05-8059-9e82e303398b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Partagé avec" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Partagé avec détails" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{91d8c4ba-4bbe-472d-8094-5353d32adf2a}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="cd07618e-4042-4e05-8059-9e82e303398b">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="cd07618e-4042-4e05-8059-9e82e303398b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557b78e-b540-44eb-8496-d55148e88a38">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <date xmlns="9557b78e-b540-44eb-8496-d55148e88a38" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69FF5FEB-3F88-44A1-8D60-295029AF89FE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C323C98-8F8D-42A2-83B1-DF821647DA0A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE3BF8E0-D9E2-4B75-B222-337A34F1BE02}"/>
 </file>
</xml_diff>